<commit_message>
Save as path dialog added, Fixes, Build related updates
</commit_message>
<xml_diff>
--- a/MM Target group.xlsx
+++ b/MM Target group.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Dr Transition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36B0F979-1DBD-4DE4-9D76-012921AB9A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2658CC51-7F66-4191-AD86-64DF9AB745DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E44257D9-226F-4616-AA04-9F48999D4D3B}"/>
   </bookViews>
@@ -719,7 +719,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2961" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3273" uniqueCount="249">
   <si>
     <t>Policy title</t>
   </si>
@@ -1415,6 +1415,57 @@
   </si>
   <si>
     <t>Energy &amp; Housing</t>
+  </si>
+  <si>
+    <t>PT_EN_AD_1</t>
+  </si>
+  <si>
+    <t>SOLENERGE</t>
+  </si>
+  <si>
+    <t>PT_EN_N_1</t>
+  </si>
+  <si>
+    <t>Accessible Zero-Emission Public Transport for All</t>
+  </si>
+  <si>
+    <t>PT_EN_N_2</t>
+  </si>
+  <si>
+    <t>Agrivoltaics Azores</t>
+  </si>
+  <si>
+    <t>PT_EN_N_3</t>
+  </si>
+  <si>
+    <t>The New Roads</t>
+  </si>
+  <si>
+    <t>PT_HO_N_1</t>
+  </si>
+  <si>
+    <t>Accessible Public Spaces</t>
+  </si>
+  <si>
+    <t>PT_HO_N_2</t>
+  </si>
+  <si>
+    <t>Integrated Neighbourhoods</t>
+  </si>
+  <si>
+    <t>PT_ENHO_N_1</t>
+  </si>
+  <si>
+    <t>Zero VAT on Energy-Efficient Equipment</t>
+  </si>
+  <si>
+    <t>PT_ENHO_N_2</t>
+  </si>
+  <si>
+    <t>Renewable Neighbourhoods</t>
+  </si>
+  <si>
+    <t>Cross-cutting (Energy &amp; Housing)</t>
   </si>
 </sst>
 </file>
@@ -1569,10 +1620,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1609,9 +1661,28 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{684F1A2B-8FE7-4201-ACD3-F793F4D306D4}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1923,7 +1994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF0A6AE8-30DB-4261-96F9-8A5E7201A3BE}">
-  <dimension ref="A1:AN76"/>
+  <dimension ref="A1:AN84"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -11072,14 +11143,960 @@
         <v>55</v>
       </c>
     </row>
+    <row r="77" spans="1:40">
+      <c r="A77" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="B77" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="C77" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D77" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="F77" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="G77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="H77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="I77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="J77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="K77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="L77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="M77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="N77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="O77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="P77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="R77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="S77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="T77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="U77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="V77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="W77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="X77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AA77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AC77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AE77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AG77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AH77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AI77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ77" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="AK77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AL77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AM77" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AN77" s="18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="78" spans="1:40">
+      <c r="A78" s="14" t="s">
+        <v>234</v>
+      </c>
+      <c r="B78" s="15" t="s">
+        <v>235</v>
+      </c>
+      <c r="C78" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D78" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="G78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="H78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="I78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="J78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="K78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="L78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="M78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="N78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="O78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="P78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="R78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="S78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="T78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="U78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="V78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="W78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="X78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AA78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AC78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AE78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AG78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AH78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AI78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AK78" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL78" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="AM78" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AN78" s="19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="79" spans="1:40">
+      <c r="A79" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="B79" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="C79" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D79" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F79" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="G79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="H79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="I79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="J79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="K79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="L79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="M79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="N79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="O79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="P79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="R79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="S79" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="T79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="U79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="V79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="W79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="X79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="Y79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AA79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AC79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="AE79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AH79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AI79" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK79" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL79" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="AM79" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="AN79" s="18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="80" spans="1:40">
+      <c r="A80" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="B80" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="C80" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D80" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F80" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="G80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="H80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="I80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="J80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="K80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="L80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="M80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="N80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="O80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="P80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="R80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="S80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="T80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="U80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="V80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="W80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="X80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AA80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AC80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD80" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="AE80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AG80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AH80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AI80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AK80" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL80" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="AM80" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AN80" s="19" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="81" spans="1:40">
+      <c r="A81" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="B81" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="C81" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D81" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="G81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="H81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="I81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="J81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="K81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="L81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="M81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="N81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="O81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="P81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="R81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="S81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="T81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="U81" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="V81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="W81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="X81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AA81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AC81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AE81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AG81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AH81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AI81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ81" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AK81" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL81" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="AM81" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="AN81" s="18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="82" spans="1:40">
+      <c r="A82" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="B82" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="C82" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D82" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F82" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="G82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="H82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="I82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="J82" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="K82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="L82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="M82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="N82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="O82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="P82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="R82" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="S82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="T82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="U82" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="V82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="W82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="X82" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="Y82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AA82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AC82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AE82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AG82" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH82" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="AI82" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="AJ82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AK82" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL82" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AM82" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="AN82" s="19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="83" spans="1:40" ht="26">
+      <c r="A83" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="B83" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="C83" s="16" t="s">
+        <v>248</v>
+      </c>
+      <c r="D83" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F83" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="G83" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="H83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="I83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="J83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="K83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="L83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="M83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="N83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="O83" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="P83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="R83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="S83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="T83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="U83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="V83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="W83" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="X83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AA83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AC83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AE83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF83" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AH83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AI83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ83" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AL83" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="AM83" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="AN83" s="18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="84" spans="1:40" ht="26">
+      <c r="A84" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="B84" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="C84" s="16" t="s">
+        <v>248</v>
+      </c>
+      <c r="D84" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F84" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="G84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="H84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="I84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="J84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="K84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="L84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="M84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="N84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="O84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="P84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="R84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="S84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="T84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="U84" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="V84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="W84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="X84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AA84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AC84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AE84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AG84" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH84" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="AI84" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="AJ84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AK84" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="AL84" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="AM84" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="AN84" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="V1:X1"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="O1:R1"/>
-    <mergeCell ref="S1:U1"/>
     <mergeCell ref="AM1:AN1"/>
     <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="AB1:AC1"/>
@@ -11087,6 +12104,12 @@
     <mergeCell ref="AF1:AH1"/>
     <mergeCell ref="AI1:AJ1"/>
     <mergeCell ref="AK1:AL1"/>
+    <mergeCell ref="V1:X1"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="O1:R1"/>
+    <mergeCell ref="S1:U1"/>
   </mergeCells>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" sqref="C3:C14" xr:uid="{BE2FA3E7-CAC1-4ECD-9C55-C1DBE1C66D95}">

</xml_diff>